<commit_message>
Nomeia João Araújo (Meta) e Gabriela Bezerra (Facebook e Instagram) nos entregáveis das tarefas 1744 e 1749
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BNtRG1wGaTmzdzTc1r8f3Q
</commit_message>
<xml_diff>
--- a/docs/nekt/inventario-fontes-1749-2026-10-15.xlsx
+++ b/docs/nekt/inventario-fontes-1749-2026-10-15.xlsx
@@ -622,7 +622,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>1. Nomear os administradores do Business Manager Meta e do MCC Google Ads. Sem nome, nenhum dos bloqueios P1 tem dono.</t>
+          <t>1. Nomear o administrador do MCC Google Ads (único sem nome; o do Business Manager Meta é João Araújo e Facebook/Instagram é Gabriela Bezerra). Sem esse nome, os bloqueios P1 do Google não têm dono.</t>
         </is>
       </c>
     </row>
@@ -709,7 +709,7 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Inventário de 15/10 + 3 linhas acrescentadas hoje (Google: Dmello, Vanguarda; Meta: nenhuma)</t>
+          <t>Inventário de 15/10 + 2 linhas acrescentadas hoje (Google: Dmello e a conta própria da Vanguarda)</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -1022,7 +1022,7 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Agendado bate em todos; excedente são execuções manuais</t>
+          <t>Agendado bate em 11 pipelines e aproximadamente no notebook; o excedente são execuções manuais</t>
         </is>
       </c>
     </row>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Sim, e estas são as razões. A planilha da #1743 dizia 71% de contas conectadas: o número é praticamente o mesmo (71,4% contra 70,9%). O one pager da #1744 dizia 101 de 159 contas com leitura validada: corrigido para 111 de 161. Motivos: a fonte da Japurá tem dado (3.189 linhas) e eu a tinha dado como sem tabela; o Google "38 validadas" contava sucesso de execução, e agora conta leitura comparada com o MCC (41); entraram duas contas Google que faltavam no inventário (Dmello e a conta própria da Vanguarda).</t>
+          <t>Sim, e estas são as razões. A planilha da #1743 dizia 71% de contas conectadas: o número é praticamente o mesmo (71,4% contra 70,9%). O one pager da #1744 dizia 101 de 159 contas com leitura validada: corrigido para 111 de 161. Motivos: a fonte da Japurá tem dado (3.189 linhas) e ela havia sido registrada como sem tabela; o Google "38 validadas" contava sucesso de execução, e agora conta leitura comparada com o MCC (41); entraram duas contas Google que faltavam no inventário (Dmello e a conta própria da Vanguarda).</t>
         </is>
       </c>
     </row>
@@ -22047,7 +22047,7 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>Aviso do conector: prazo de 23/10/2026. A Nekt marca "vencido" como falso hoje.</t>
+          <t>Aviso do conector: prazo de 23/10/2026. O indicador de vencimento da Nekt ainda mostra "não vencido".</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
@@ -22124,7 +22124,7 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Admin do Business Manager Meta (nome a confirmar)</t>
+          <t>João Araújo (admin Meta)</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -22191,7 +22191,7 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Admin do Business Manager Meta + Jussara</t>
+          <t>João Araújo (admin Meta) + Jussara</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
@@ -22325,7 +22325,7 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Suporte Nekt + Admin do Business Manager</t>
+          <t>Suporte Nekt + João Araújo (admin Meta)</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -22526,7 +22526,7 @@
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>João (mapeamento)</t>
+          <t>João Araújo (mapeamento)</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
@@ -22861,7 +22861,7 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>Jussara + Social Media</t>
+          <t>Gabriela Bezerra (Facebook e Instagram) + Jussara</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
@@ -23601,7 +23601,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Admin do BM Meta; Admin do MCC Google; gestor de mídia; suporte Nekt</t>
+          <t>João Araújo (BM Meta); Admin do MCC Google (a confirmar); gestor de mídia; suporte Nekt</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -23643,7 +23643,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Admin do BM; Admin do MCC; AMs; analistas Inbound; Jussara (camadas)</t>
+          <t>João Araújo (BM Meta); Admin do MCC (a confirmar); AMs; analistas Inbound; Jussara (camadas)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -23727,7 +23727,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>João e analistas; admins das contas</t>
+          <t>João Araújo e analistas; admins das contas</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -23769,7 +23769,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Jussara + Social Media</t>
+          <t>Gabriela Bezerra (Facebook e Instagram) + Jussara</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">

</xml_diff>